<commit_message>
implementacion de barras de progresp y listado de pasajeros
</commit_message>
<xml_diff>
--- a/data/output/pasajeros_geocodificados.xlsx
+++ b/data/output/pasajeros_geocodificados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,11 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>nota_precision</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>error_detalle</t>
         </is>
       </c>
@@ -497,6 +502,7 @@
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -532,6 +538,7 @@
         </is>
       </c>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -552,14 +559,14 @@
       <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Calle 30 #22-18, Soledad, Atlantico</t>
+          <t>Calle 30 #22-18, Soledad, Atlántico</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>10.9370509</v>
+        <v>10.9336875</v>
       </c>
       <c r="G4" t="n">
-        <v>-74.7752338</v>
+        <v>-74.7767353</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -567,6 +574,7 @@
         </is>
       </c>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -591,10 +599,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>10.866502</v>
+        <v>10.8679568</v>
       </c>
       <c r="G5" t="n">
-        <v>-74.7737643</v>
+        <v>-74.7792501</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -602,6 +610,7 @@
         </is>
       </c>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -637,6 +646,7 @@
         </is>
       </c>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -676,6 +686,7 @@
         </is>
       </c>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>